<commit_message>
MI workflow stabilization and badge engine fixes
- Status engine reordered and corrected
- Completion removal rollback implemented
- Permission-driven auto transitions fixed
- Doc state entity mapping corrected
- Serializer field alignment
- Dropdown preload bug resolved
- Detail page state handling improved
</commit_message>
<xml_diff>
--- a/docs/ARCAD_System_Library.xlsx
+++ b/docs/ARCAD_System_Library.xlsx
@@ -5,17 +5,18 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahidakhtar/ARCAD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahidakhtar/ARCAD/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6C1B4C4-CCD3-3942-BA20-0C5E0A87885D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C31871EF-F2A6-B344-96C2-FA0ABD1611DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="9520" windowWidth="30240" windowHeight="8920" xr2:uid="{D3E83B99-027E-4143-A195-C99C62BA1DBF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{D3E83B99-027E-4143-A195-C99C62BA1DBF}"/>
   </bookViews>
   <sheets>
     <sheet name="d1" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="115">
   <si>
     <t>invoice</t>
   </si>
@@ -176,108 +177,72 @@
     <t>Open</t>
   </si>
   <si>
-    <t>#ADD8E6</t>
-  </si>
-  <si>
     <t>perm_wait</t>
   </si>
   <si>
     <t>Permission Awaited</t>
   </si>
   <si>
-    <t>#FFE5B4</t>
-  </si>
-  <si>
     <t>perm_issue</t>
   </si>
   <si>
     <t>Permission Issue</t>
   </si>
   <si>
-    <t>#FFA500</t>
-  </si>
-  <si>
     <t>appr_wait</t>
   </si>
   <si>
     <t>Approval Awaited</t>
   </si>
   <si>
-    <t>#E6F2FF</t>
-  </si>
-  <si>
     <t>hold</t>
   </si>
   <si>
     <t>Hold</t>
   </si>
   <si>
-    <t>#FFD700</t>
-  </si>
-  <si>
     <t>down</t>
   </si>
   <si>
     <t>Down</t>
   </si>
   <si>
-    <t>#FF0000</t>
-  </si>
-  <si>
     <t>live</t>
   </si>
   <si>
     <t>Live</t>
   </si>
   <si>
-    <t>#008000</t>
-  </si>
-  <si>
     <t>term</t>
   </si>
   <si>
     <t>Terminated</t>
   </si>
   <si>
-    <t>#FF8C00</t>
-  </si>
-  <si>
     <t>rect</t>
   </si>
   <si>
     <t>Rectification</t>
   </si>
   <si>
-    <t>#E8FFE8</t>
-  </si>
-  <si>
     <t>cancel</t>
   </si>
   <si>
     <t>Cancelled</t>
   </si>
   <si>
-    <t>#FFCCCC</t>
-  </si>
-  <si>
     <t>comp</t>
   </si>
   <si>
     <t>Completed</t>
   </si>
   <si>
-    <t>#CCFFCC</t>
-  </si>
-  <si>
     <t>staged</t>
   </si>
   <si>
     <t>Staged</t>
   </si>
   <si>
-    <t>#808080</t>
-  </si>
-  <si>
     <t>doc_state</t>
   </si>
   <si>
@@ -305,9 +270,6 @@
     <t>Rejected</t>
   </si>
   <si>
-    <t>#FF9999</t>
-  </si>
-  <si>
     <t>badge_entity_map</t>
   </si>
   <si>
@@ -375,12 +337,60 @@
   </si>
   <si>
     <t>badge_id (FK, not null)</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>#0AACE8</t>
+  </si>
+  <si>
+    <t>#93DCF9</t>
+  </si>
+  <si>
+    <t>#F1CA00</t>
+  </si>
+  <si>
+    <t>#FEFE01</t>
+  </si>
+  <si>
+    <t>#FD0000</t>
+  </si>
+  <si>
+    <t>#92D050</t>
+  </si>
+  <si>
+    <t>#F3C214</t>
+  </si>
+  <si>
+    <t>#E3EDD2</t>
+  </si>
+  <si>
+    <t>#F2D0D3</t>
+  </si>
+  <si>
+    <t>#7F7F7F</t>
+  </si>
+  <si>
+    <t>Job</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>unit cost</t>
+  </si>
+  <si>
+    <t>mast installation</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -403,7 +413,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -418,55 +428,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFADD8E6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFE5B4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFA500"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE6F2FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFD700"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF008000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF8C00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8FFE8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -478,24 +440,42 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCCFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF808080"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF9999"/>
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -518,11 +498,81 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -533,55 +583,64 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -919,7 +978,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918BE53B-16EF-6F47-8F4B-48571349F3F8}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:R43"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" style="1" customWidth="1"/>
@@ -929,90 +988,93 @@
     <col min="6" max="6" width="12.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" style="1"/>
+    <col min="9" max="9" width="10.83203125" style="14"/>
     <col min="10" max="11" width="10.83203125" style="1"/>
     <col min="12" max="12" width="21.83203125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="10.83203125" style="1"/>
-    <col min="15" max="15" width="13.1640625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="14.33203125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" style="1"/>
-    <col min="18" max="18" width="10.83203125" style="19"/>
-    <col min="19" max="16384" width="10.83203125" style="1"/>
+    <col min="15" max="15" width="10.83203125" style="1"/>
+    <col min="16" max="16" width="13.1640625" style="1" customWidth="1"/>
+    <col min="17" max="17" width="14.33203125" style="1" customWidth="1"/>
+    <col min="18" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:19" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="D1" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="J1" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="N1" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="D1" s="4" t="s">
+      <c r="O1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="R1" s="11"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="1:19" ht="51" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="J1" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="N1" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="20"/>
-    </row>
-    <row r="2" spans="1:18" ht="51" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="J2" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="L2" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>110</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="N2" s="12"/>
       <c r="O2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="Q2" s="5"/>
-      <c r="R2" s="20"/>
-    </row>
-    <row r="3" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="6"/>
+    </row>
+    <row r="3" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -1027,7 +1089,7 @@
         <v>18</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J3" s="3">
         <v>1</v>
@@ -1042,22 +1104,26 @@
         <v>10</v>
       </c>
       <c r="O3" s="3">
-        <f>_xlfn.XLOOKUP(Q3, F$3:F$34, D$3:D$34)</f>
+        <f>_xlfn.XLOOKUP(N3, K$3:K$10, J$3:J$10)</f>
         <v>1</v>
       </c>
-      <c r="P3" s="3" t="s">
+      <c r="P3" s="3">
+        <f>_xlfn.XLOOKUP(R3, F$3:F$34, D$3:D$34)</f>
+        <v>1</v>
+      </c>
+      <c r="Q3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="3" t="s">
+      <c r="R3" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
@@ -1072,7 +1138,7 @@
         <v>20</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J4" s="3">
         <v>2</v>
@@ -1087,22 +1153,26 @@
         <v>10</v>
       </c>
       <c r="O4" s="3">
-        <f t="shared" ref="O4:O43" si="0">_xlfn.XLOOKUP(Q4, F$3:F$34, D$3:D$34)</f>
+        <f t="shared" ref="O4:O43" si="0">_xlfn.XLOOKUP(N4, K$3:K$10, J$3:J$10)</f>
+        <v>1</v>
+      </c>
+      <c r="P4" s="3">
+        <f t="shared" ref="P4:P43" si="1">_xlfn.XLOOKUP(R4, F$3:F$34, D$3:D$34)</f>
         <v>2</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="R4" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="D5" s="3">
         <v>3</v>
@@ -1117,7 +1187,7 @@
         <v>22</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J5" s="3">
         <v>3</v>
@@ -1133,21 +1203,25 @@
       </c>
       <c r="O5" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P5" s="3">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="P5" s="3" t="s">
+      <c r="Q5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="3" t="s">
+      <c r="R5" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
@@ -1162,7 +1236,7 @@
         <v>24</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J6" s="3">
         <v>4</v>
@@ -1178,21 +1252,25 @@
       </c>
       <c r="O6" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P6" s="3">
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="P6" s="3" t="s">
+      <c r="Q6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q6" s="3" t="s">
+      <c r="R6" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="D7" s="3">
         <v>5</v>
@@ -1207,7 +1285,7 @@
         <v>26</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J7" s="3">
         <v>5</v>
@@ -1223,16 +1301,20 @@
       </c>
       <c r="O7" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P7" s="3">
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="P7" s="3" t="s">
+      <c r="Q7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q7" s="3" t="s">
+      <c r="R7" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D8" s="3">
         <v>6</v>
       </c>
@@ -1246,7 +1328,7 @@
         <v>29</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J8" s="3">
         <v>6</v>
@@ -1262,16 +1344,20 @@
       </c>
       <c r="O8" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P8" s="3">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="P8" s="3" t="s">
+      <c r="Q8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Q8" s="3" t="s">
+      <c r="R8" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D9" s="3">
         <v>7</v>
       </c>
@@ -1285,7 +1371,7 @@
         <v>31</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J9" s="3">
         <v>7</v>
@@ -1301,16 +1387,20 @@
       </c>
       <c r="O9" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P9" s="3">
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
-      <c r="P9" s="3" t="s">
+      <c r="Q9" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Q9" s="3" t="s">
+      <c r="R9" s="3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D10" s="3">
         <v>8</v>
       </c>
@@ -1324,7 +1414,7 @@
         <v>33</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="J10" s="3">
         <v>8</v>
@@ -1340,16 +1430,20 @@
       </c>
       <c r="O10" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P10" s="3">
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="Q10" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Q10" s="3" t="s">
+      <c r="R10" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D11" s="3">
         <v>9</v>
       </c>
@@ -1363,23 +1457,27 @@
         <v>35</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="N11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="O11" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P11" s="3">
+        <f t="shared" si="1"/>
         <v>9</v>
       </c>
-      <c r="P11" s="3" t="s">
+      <c r="Q11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Q11" s="3" t="s">
+      <c r="R11" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D12" s="3">
         <v>12</v>
       </c>
@@ -1393,23 +1491,27 @@
         <v>37</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="N12" s="3" t="s">
         <v>10</v>
       </c>
       <c r="O12" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P12" s="3">
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="P12" s="3" t="s">
+      <c r="Q12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="Q12" s="3" t="s">
+      <c r="R12" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
       <c r="D13" s="3">
         <v>10</v>
       </c>
@@ -1423,23 +1525,27 @@
         <v>40</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="N13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="O13" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P13" s="3">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="P13" s="3" t="s">
+      <c r="Q13" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="Q13" s="3" t="s">
+      <c r="R13" s="3" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="D14" s="3">
         <v>11</v>
       </c>
@@ -1453,23 +1559,27 @@
         <v>42</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>101</v>
+        <v>88</v>
       </c>
       <c r="N14" s="3" t="s">
         <v>10</v>
       </c>
       <c r="O14" s="3">
         <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="P14" s="3">
+        <f t="shared" si="1"/>
         <v>11</v>
       </c>
-      <c r="P14" s="3" t="s">
+      <c r="Q14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="Q14" s="3" t="s">
+      <c r="R14" s="3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D15" s="3">
         <v>13</v>
       </c>
@@ -1482,24 +1592,28 @@
       <c r="G15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H15" s="6" t="s">
-        <v>46</v>
+      <c r="H15" s="15" t="s">
+        <v>101</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O15" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P15" s="3">
+        <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="P15" s="3" t="s">
+      <c r="Q15" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q15" s="3" t="s">
+      <c r="R15" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="D16" s="3">
         <v>14</v>
       </c>
@@ -1507,29 +1621,33 @@
         <v>43</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>49</v>
+      <c r="H16" s="16" t="s">
+        <v>102</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O16" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P16" s="3">
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
-      <c r="P16" s="3" t="s">
+      <c r="Q16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q16" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="4:17" ht="34" x14ac:dyDescent="0.2">
+      <c r="R16" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="4:18" ht="34" x14ac:dyDescent="0.2">
       <c r="D17" s="3">
         <v>15</v>
       </c>
@@ -1537,29 +1655,33 @@
         <v>43</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>103</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O17" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P17" s="3">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="P17" s="3" t="s">
+      <c r="Q17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q17" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="4:17" ht="34" x14ac:dyDescent="0.2">
+      <c r="R17" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" spans="4:18" ht="34" x14ac:dyDescent="0.2">
       <c r="D18" s="3">
         <v>16</v>
       </c>
@@ -1567,29 +1689,33 @@
         <v>43</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H18" s="9" t="s">
-        <v>55</v>
+        <v>51</v>
+      </c>
+      <c r="H18" s="18" t="s">
+        <v>104</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O18" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P18" s="3">
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
-      <c r="P18" s="3" t="s">
+      <c r="Q18" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q18" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R18" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D19" s="3">
         <v>17</v>
       </c>
@@ -1597,29 +1723,33 @@
         <v>43</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>58</v>
+        <v>53</v>
+      </c>
+      <c r="H19" s="18" t="s">
+        <v>104</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O19" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P19" s="3">
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="P19" s="3" t="s">
+      <c r="Q19" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q19" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="20" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R19" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D20" s="3">
         <v>18</v>
       </c>
@@ -1627,29 +1757,33 @@
         <v>43</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>61</v>
+        <v>55</v>
+      </c>
+      <c r="H20" s="19" t="s">
+        <v>105</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O20" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P20" s="3">
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="P20" s="3" t="s">
+      <c r="Q20" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q20" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="21" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R20" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D21" s="3">
         <v>19</v>
       </c>
@@ -1657,29 +1791,33 @@
         <v>43</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>64</v>
+        <v>57</v>
+      </c>
+      <c r="H21" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O21" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P21" s="3">
+        <f t="shared" si="1"/>
         <v>19</v>
       </c>
-      <c r="P21" s="3" t="s">
+      <c r="Q21" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q21" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R21" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D22" s="3">
         <v>20</v>
       </c>
@@ -1687,29 +1825,33 @@
         <v>43</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="H22" s="13" t="s">
-        <v>67</v>
+        <v>59</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>107</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O22" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P22" s="3">
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="P22" s="3" t="s">
+      <c r="Q22" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q22" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R22" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="23" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D23" s="3">
         <v>21</v>
       </c>
@@ -1717,29 +1859,33 @@
         <v>43</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="H23" s="14" t="s">
-        <v>70</v>
+        <v>61</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>108</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O23" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P23" s="3">
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
-      <c r="P23" s="3" t="s">
+      <c r="Q23" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q23" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R23" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D24" s="3">
         <v>22</v>
       </c>
@@ -1747,29 +1893,33 @@
         <v>43</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>73</v>
+        <v>63</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="N24" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O24" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P24" s="3">
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
-      <c r="P24" s="3" t="s">
+      <c r="Q24" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q24" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R24" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D25" s="3">
         <v>23</v>
       </c>
@@ -1777,29 +1927,33 @@
         <v>43</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="H25" s="16" t="s">
-        <v>76</v>
+        <v>65</v>
+      </c>
+      <c r="H25" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O25" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P25" s="3">
+        <f t="shared" si="1"/>
         <v>23</v>
       </c>
-      <c r="P25" s="3" t="s">
+      <c r="Q25" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q25" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R25" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D26" s="3">
         <v>24</v>
       </c>
@@ -1807,411 +1961,530 @@
         <v>43</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="H26" s="17" t="s">
-        <v>79</v>
+        <v>67</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="N26" s="3" t="s">
         <v>11</v>
       </c>
       <c r="O26" s="3">
         <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="P26" s="3">
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="P26" s="3" t="s">
+      <c r="Q26" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="Q26" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+      <c r="R26" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D27" s="3">
         <v>25</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>6</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H27" s="15" t="s">
-        <v>73</v>
+        <v>69</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>109</v>
       </c>
       <c r="N27" s="3" t="s">
         <v>12</v>
       </c>
       <c r="O27" s="3">
         <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="P27" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P27" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q27" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R27" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="28" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D28" s="3">
         <v>26</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>9</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H28" s="16" t="s">
-        <v>76</v>
+        <v>70</v>
+      </c>
+      <c r="H28" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>12</v>
       </c>
       <c r="O28" s="3">
         <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="P28" s="3">
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
-      <c r="P28" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q28" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R28" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D29" s="3">
         <v>27</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="H29" s="9" t="s">
-        <v>55</v>
+        <v>71</v>
+      </c>
+      <c r="H29" s="14" t="s">
+        <v>102</v>
       </c>
       <c r="N29" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O29" s="3">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P29" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P29" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q29" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R29" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="30" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D30" s="3">
         <v>28</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>2</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>46</v>
+        <v>72</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>101</v>
       </c>
       <c r="N30" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O30" s="3">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P30" s="3">
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="P30" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q30" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R30" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="31" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D31" s="3">
         <v>29</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>8</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H31" s="12" t="s">
-        <v>64</v>
+        <v>73</v>
+      </c>
+      <c r="H31" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N31" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O31" s="3">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P31" s="3">
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="P31" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q31" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R31" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D32" s="3">
         <v>30</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>3</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="H32" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="H32" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N32" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O32" s="3">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P32" s="3">
+        <f t="shared" si="1"/>
         <v>39</v>
       </c>
-      <c r="P32" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q32" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R32" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="33" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D33" s="3">
         <v>31</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="H33" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="H33" s="20" t="s">
+        <v>106</v>
       </c>
       <c r="N33" s="3" t="s">
         <v>0</v>
       </c>
       <c r="O33" s="3">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P33" s="3">
+        <f t="shared" si="1"/>
         <v>29</v>
       </c>
-      <c r="P33" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q33" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R33" s="3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="34" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D34" s="3">
         <v>39</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="F34" s="3" t="s">
         <v>5</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="H34" s="18" t="s">
-        <v>89</v>
+        <v>76</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>105</v>
       </c>
       <c r="N34" s="3" t="s">
         <v>1</v>
       </c>
       <c r="O34" s="3">
         <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="P34" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P34" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q34" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R34" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="35" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N35" s="3" t="s">
         <v>1</v>
       </c>
       <c r="O35" s="3">
         <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="P35" s="3">
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="P35" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q35" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R35" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="36" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N36" s="3" t="s">
         <v>13</v>
       </c>
       <c r="O36" s="3">
         <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="P36" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P36" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q36" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R36" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N37" s="3" t="s">
         <v>13</v>
       </c>
       <c r="O37" s="3">
         <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="P37" s="3">
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="P37" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q37" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R37" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N38" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O38" s="3">
         <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="P38" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P38" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R38" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="39" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N39" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O39" s="3">
         <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="P39" s="3">
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="P39" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q39" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R39" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="40" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N40" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O40" s="3">
         <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="P40" s="3">
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="P40" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q40" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R40" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="41" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N41" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O41" s="3">
         <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P41" s="3">
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="P41" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q41" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R41" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="42" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N42" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O42" s="3">
         <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P42" s="3">
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
-      <c r="P42" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q42" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R42" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="4:17" ht="17" x14ac:dyDescent="0.2">
+    <row r="43" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="N43" s="3" t="s">
         <v>15</v>
       </c>
       <c r="O43" s="3">
         <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="P43" s="3">
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
-      <c r="P43" s="3" t="s">
-        <v>80</v>
-      </c>
       <c r="Q43" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="R43" s="3" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="Q1:R2"/>
+    <mergeCell ref="N1:N2"/>
     <mergeCell ref="J1:L1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:H1"/>
-    <mergeCell ref="P2:Q2"/>
-    <mergeCell ref="N1:Q1"/>
+    <mergeCell ref="O1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5887C558-A2C5-BF4A-B57F-FF058A42D75F}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B2" s="22">
+        <v>36526</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" s="23">
+        <v>46044</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2600</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Stabilize badge engine, remove hardcoded entity_type, add is_manual, fix volume + healthcheck, restore transitions
</commit_message>
<xml_diff>
--- a/docs/ARCAD_System_Library.xlsx
+++ b/docs/ARCAD_System_Library.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahidakhtar/ARCAD/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C31871EF-F2A6-B344-96C2-FA0ABD1611DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F543BE9F-063A-6C43-91BB-64965EE7E5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{D3E83B99-027E-4143-A195-C99C62BA1DBF}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{D3E83B99-027E-4143-A195-C99C62BA1DBF}"/>
   </bookViews>
   <sheets>
     <sheet name="d1" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="119">
   <si>
     <t>invoice</t>
   </si>
@@ -382,6 +382,18 @@
   </si>
   <si>
     <t>mast installation</t>
+  </si>
+  <si>
+    <t>project_id</t>
+  </si>
+  <si>
+    <t>from</t>
+  </si>
+  <si>
+    <t>to</t>
+  </si>
+  <si>
+    <t>entity type id</t>
   </si>
 </sst>
 </file>
@@ -389,7 +401,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -592,27 +604,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -637,10 +628,31 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -988,7 +1000,7 @@
     <col min="6" max="6" width="12.6640625" style="1" customWidth="1"/>
     <col min="7" max="7" width="12.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="10.83203125" style="1"/>
-    <col min="9" max="9" width="10.83203125" style="14"/>
+    <col min="9" max="9" width="10.83203125" style="7"/>
     <col min="10" max="11" width="10.83203125" style="1"/>
     <col min="12" max="12" width="21.83203125" style="1" customWidth="1"/>
     <col min="15" max="15" width="10.83203125" style="1"/>
@@ -998,33 +1010,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="D1" s="7" t="s">
+      <c r="B1" s="21"/>
+      <c r="D1" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="J1" s="7" t="s">
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="J1" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="N1" s="10" t="s">
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="N1" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="O1" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="P1" s="9"/>
-      <c r="Q1" s="10" t="s">
+      <c r="P1" s="23"/>
+      <c r="Q1" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="R1" s="11"/>
+      <c r="R1" s="18"/>
       <c r="S1" s="6"/>
     </row>
     <row r="2" spans="1:19" ht="51" x14ac:dyDescent="0.2">
@@ -1058,18 +1070,18 @@
       <c r="L2" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="N2" s="12"/>
+      <c r="N2" s="19"/>
       <c r="O2" s="2" t="s">
         <v>97</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="13"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="20"/>
       <c r="S2" s="6"/>
     </row>
-    <row r="3" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>78</v>
       </c>
@@ -1118,7 +1130,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>79</v>
       </c>
@@ -1167,7 +1179,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>77</v>
       </c>
@@ -1216,7 +1228,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
@@ -1265,7 +1277,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
@@ -1314,7 +1326,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D8" s="3">
         <v>6</v>
       </c>
@@ -1357,7 +1369,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D9" s="3">
         <v>7</v>
       </c>
@@ -1400,7 +1412,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D10" s="3">
         <v>8</v>
       </c>
@@ -1443,7 +1455,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D11" s="3">
         <v>9</v>
       </c>
@@ -1477,7 +1489,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D12" s="3">
         <v>12</v>
       </c>
@@ -1511,7 +1523,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:19" ht="17" x14ac:dyDescent="0.2">
       <c r="D13" s="3">
         <v>10</v>
       </c>
@@ -1545,7 +1557,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:19" ht="34" x14ac:dyDescent="0.2">
       <c r="D14" s="3">
         <v>11</v>
       </c>
@@ -1592,8 +1604,20 @@
       <c r="G15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H15" s="15" t="s">
+      <c r="H15" s="8" t="s">
         <v>101</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="N15" s="3" t="s">
         <v>11</v>
@@ -1626,8 +1650,20 @@
       <c r="G16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="H16" s="16" t="s">
+      <c r="H16" s="9" t="s">
         <v>102</v>
+      </c>
+      <c r="I16" s="7">
+        <v>2</v>
+      </c>
+      <c r="J16" s="1">
+        <v>1</v>
+      </c>
+      <c r="K16" s="1">
+        <v>13</v>
+      </c>
+      <c r="L16" s="1">
+        <v>17</v>
       </c>
       <c r="N16" s="3" t="s">
         <v>11</v>
@@ -1660,8 +1696,20 @@
       <c r="G17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="10" t="s">
         <v>103</v>
+      </c>
+      <c r="I17" s="7">
+        <v>2</v>
+      </c>
+      <c r="J17" s="1">
+        <v>1</v>
+      </c>
+      <c r="K17" s="1">
+        <v>13</v>
+      </c>
+      <c r="L17" s="1">
+        <v>22</v>
       </c>
       <c r="N17" s="3" t="s">
         <v>11</v>
@@ -1694,8 +1742,20 @@
       <c r="G18" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="H18" s="11" t="s">
         <v>104</v>
+      </c>
+      <c r="I18" s="7">
+        <v>2</v>
+      </c>
+      <c r="J18" s="1">
+        <v>1</v>
+      </c>
+      <c r="K18" s="1">
+        <v>17</v>
+      </c>
+      <c r="L18" s="1">
+        <v>14</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>11</v>
@@ -1728,8 +1788,20 @@
       <c r="G19" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="H19" s="11" t="s">
         <v>104</v>
+      </c>
+      <c r="I19" s="7">
+        <v>2</v>
+      </c>
+      <c r="J19" s="1">
+        <v>1</v>
+      </c>
+      <c r="K19" s="1">
+        <v>17</v>
+      </c>
+      <c r="L19" s="1">
+        <v>22</v>
       </c>
       <c r="N19" s="3" t="s">
         <v>11</v>
@@ -1762,8 +1834,20 @@
       <c r="G20" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="H20" s="19" t="s">
+      <c r="H20" s="12" t="s">
         <v>105</v>
+      </c>
+      <c r="I20" s="7">
+        <v>2</v>
+      </c>
+      <c r="J20" s="1">
+        <v>1</v>
+      </c>
+      <c r="K20" s="1">
+        <v>22</v>
+      </c>
+      <c r="L20" s="1">
+        <v>17</v>
       </c>
       <c r="N20" s="3" t="s">
         <v>11</v>
@@ -1796,8 +1880,20 @@
       <c r="G21" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="H21" s="20" t="s">
+      <c r="H21" s="13" t="s">
         <v>106</v>
+      </c>
+      <c r="I21" s="7">
+        <v>2</v>
+      </c>
+      <c r="J21" s="1">
+        <v>1</v>
+      </c>
+      <c r="K21" s="1">
+        <v>22</v>
+      </c>
+      <c r="L21" s="1">
+        <v>14</v>
       </c>
       <c r="N21" s="3" t="s">
         <v>11</v>
@@ -1830,8 +1926,14 @@
       <c r="G22" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="H22" s="17" t="s">
+      <c r="H22" s="10" t="s">
         <v>107</v>
+      </c>
+      <c r="I22" s="7">
+        <v>3</v>
+      </c>
+      <c r="J22" s="1">
+        <v>1</v>
       </c>
       <c r="N22" s="3" t="s">
         <v>11</v>
@@ -1864,8 +1966,14 @@
       <c r="G23" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="H23" s="21" t="s">
+      <c r="H23" s="14" t="s">
         <v>108</v>
+      </c>
+      <c r="I23" s="7">
+        <v>2</v>
+      </c>
+      <c r="J23" s="1">
+        <v>1</v>
       </c>
       <c r="N23" s="3" t="s">
         <v>11</v>
@@ -1901,6 +2009,12 @@
       <c r="H24" s="4" t="s">
         <v>109</v>
       </c>
+      <c r="I24" s="7">
+        <v>2</v>
+      </c>
+      <c r="J24" s="1">
+        <v>1</v>
+      </c>
       <c r="N24" s="3" t="s">
         <v>11</v>
       </c>
@@ -1932,8 +2046,14 @@
       <c r="G25" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="H25" s="13" t="s">
         <v>106</v>
+      </c>
+      <c r="I25" s="7">
+        <v>2</v>
+      </c>
+      <c r="J25" s="1">
+        <v>1</v>
       </c>
       <c r="N25" s="3" t="s">
         <v>11</v>
@@ -1969,6 +2089,12 @@
       <c r="H26" s="5" t="s">
         <v>110</v>
       </c>
+      <c r="I26" s="7">
+        <v>2</v>
+      </c>
+      <c r="J26" s="1">
+        <v>1</v>
+      </c>
       <c r="N26" s="3" t="s">
         <v>11</v>
       </c>
@@ -2003,6 +2129,12 @@
       <c r="H27" s="4" t="s">
         <v>109</v>
       </c>
+      <c r="I27" s="7">
+        <v>2</v>
+      </c>
+      <c r="J27" s="1">
+        <v>1</v>
+      </c>
       <c r="N27" s="3" t="s">
         <v>12</v>
       </c>
@@ -2034,8 +2166,14 @@
       <c r="G28" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="H28" s="20" t="s">
+      <c r="H28" s="13" t="s">
         <v>106</v>
+      </c>
+      <c r="I28" s="7">
+        <v>2</v>
+      </c>
+      <c r="J28" s="1">
+        <v>1</v>
       </c>
       <c r="N28" s="3" t="s">
         <v>12</v>
@@ -2068,7 +2206,7 @@
       <c r="G29" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="14" t="s">
+      <c r="H29" s="7" t="s">
         <v>102</v>
       </c>
       <c r="N29" s="3" t="s">
@@ -2102,7 +2240,7 @@
       <c r="G30" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="H30" s="15" t="s">
+      <c r="H30" s="8" t="s">
         <v>101</v>
       </c>
       <c r="N30" s="3" t="s">
@@ -2136,7 +2274,7 @@
       <c r="G31" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="H31" s="20" t="s">
+      <c r="H31" s="13" t="s">
         <v>106</v>
       </c>
       <c r="N31" s="3" t="s">
@@ -2170,7 +2308,7 @@
       <c r="G32" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="H32" s="20" t="s">
+      <c r="H32" s="13" t="s">
         <v>106</v>
       </c>
       <c r="N32" s="3" t="s">
@@ -2182,7 +2320,7 @@
       </c>
       <c r="P32" s="3">
         <f t="shared" si="1"/>
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="Q32" s="3" t="s">
         <v>68</v>
@@ -2204,7 +2342,7 @@
       <c r="G33" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="H33" s="20" t="s">
+      <c r="H33" s="13" t="s">
         <v>106</v>
       </c>
       <c r="N33" s="3" t="s">
@@ -2227,7 +2365,7 @@
     </row>
     <row r="34" spans="4:18" ht="17" x14ac:dyDescent="0.2">
       <c r="D34" s="3">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>68</v>
@@ -2238,7 +2376,7 @@
       <c r="G34" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="H34" s="19" t="s">
+      <c r="H34" s="12" t="s">
         <v>105</v>
       </c>
       <c r="N34" s="3" t="s">
@@ -2466,7 +2604,7 @@
       <c r="A2" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B2" s="22">
+      <c r="B2" s="15">
         <v>36526</v>
       </c>
       <c r="C2" s="1">
@@ -2477,7 +2615,7 @@
       <c r="A3" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="16">
         <v>46044</v>
       </c>
       <c r="C3" s="1">

</xml_diff>

<commit_message>
Initial commit - ARCAD full stack setup
</commit_message>
<xml_diff>
--- a/docs/ARCAD_System_Library.xlsx
+++ b/docs/ARCAD_System_Library.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wahidakhtar/ARCAD/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F543BE9F-063A-6C43-91BB-64965EE7E5D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{668CA085-69B5-ED45-810A-893E6F5C9490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" xr2:uid="{D3E83B99-027E-4143-A195-C99C62BA1DBF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="120">
   <si>
     <t>invoice</t>
   </si>
@@ -394,6 +394,9 @@
   </si>
   <si>
     <t>entity type id</t>
+  </si>
+  <si>
+    <t>l3</t>
   </si>
 </sst>
 </file>
@@ -990,7 +993,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918BE53B-16EF-6F47-8F4B-48571349F3F8}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A1:S44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.1640625" style="1" customWidth="1"/>
@@ -2566,6 +2569,24 @@
       </c>
       <c r="R43" s="3" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="4:18" ht="17" x14ac:dyDescent="0.2">
+      <c r="N44" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="O44" s="3">
+        <f t="shared" ref="O44" si="2">_xlfn.XLOOKUP(N44, K$3:K$10, J$3:J$10)</f>
+        <v>1</v>
+      </c>
+      <c r="P44" s="3">
+        <v>33</v>
+      </c>
+      <c r="Q44" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="R44" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>